<commit_message>
docs(qa): Review phases 0-6, fix traceability and no-verdict gaps
Copilot-review findings resolved: BUG-LEAVE-001 converted to an
explicitly unfilled template (correct TC-LEAVE-005 link and evidence
path); RTM ranges aligned to the authored suite and string-None
defect cells cleared; DRS LEAVE-003 probe mapping aligned;
execution workbook pre-filled with 54 Not-Run rows matching suite
IDs; test summary rewritten with actual env and not-started status;
LICENSE added; exploratory session/findings stubs added.
</commit_message>
<xml_diff>
--- a/docs/05-traceability/rtm.xlsx
+++ b/docs/05-traceability/rtm.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>TC-PIM-004–007</t>
+          <t>TC-PIM-004–006, TC-PIM-009–010</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TC-PIM-008–009</t>
+          <t>TC-PIM-007–008</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>TC-LEAVE-002–004, TC-LEAVE-008</t>
+          <t>TC-LEAVE-002–004</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>TC-LEAVE-005</t>
+          <t>TC-LEAVE-005–006 (006 = past-date policy probe)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>TC-LEAVE-006–007</t>
+          <t>TC-LEAVE-007–008</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(qa): Clear execution entry gates on pinned 5.8.1 build
Complete the installer (host networking after bridge TCP timeout,
existing DB, 168 tables), provision qa_admin + qa_ess with verified
logins, verify 12-module role nav (Reports partial, no top-level),
resolve RTM Time/Recruitment conditionals, and refresh stale
pending-auth language across README, plan, inventory, and env record.
TEST-CYCLE-01 entry gates now all clear.
</commit_message>
<xml_diff>
--- a/docs/05-traceability/rtm.xlsx
+++ b/docs/05-traceability/rtm.xlsx
@@ -1003,7 +1003,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Conditional: Time presence</t>
+          <t>Present (verified in nav 2026-10-03)</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Conditional: Recruitment presence</t>
+          <t>Present, admin-side (verified in nav 2026-10-03)</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Conditional: Reports presence</t>
+          <t>Partial: sub-views under PIM/Leave/Time; confirm per-case in execution</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qa): Complete phases 7-10 RTM gate, smoke, discovery, regression
</commit_message>
<xml_diff>
--- a/docs/05-traceability/rtm.xlsx
+++ b/docs/05-traceability/rtm.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>TC-AUTH-007–008</t>
+          <t>TC-AUTH-007, TC-AUTH-008, TC-DASH-004</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>TC-DASH-001–004</t>
+          <t>TC-DASH-001–003</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TC-PIM-001</t>
+          <t>TC-PIM-001, TC-PIM-003</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>TC-PIM-002–003</t>
+          <t>TC-PIM-002</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(qa): Clarify executed requirement coverage and evidence links
</commit_message>
<xml_diff>
--- a/docs/05-traceability/rtm.xlsx
+++ b/docs/05-traceability/rtm.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1 Fail; 1 Blocked</t>
+          <t>1 Pass; 1 Fail</t>
         </is>
       </c>
       <c r="E7" s="2" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2 Blocked; 3 Not Run</t>
+          <t>2 Pass; 3 Not Run</t>
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
@@ -728,7 +728,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>1 Blocked; 1 Not Run</t>
+          <t>1 Pass; 1 Not Run</t>
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
@@ -761,7 +761,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1 Blocked</t>
+          <t>1 Pass</t>
         </is>
       </c>
       <c r="E10" s="2" t="n"/>

</xml_diff>